<commit_message>
Improve July schedule Excel with personal sheets per driver
Co-authored-by: gltdelete-prog <gltdelete-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SERDECHNOV-grafik-20-31-iyulya-2026.xlsx
+++ b/SERDECHNOV-grafik-20-31-iyulya-2026.xlsx
@@ -10,6 +10,9 @@
     <sheet name="График 20-31 июля" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Зарплата" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="График 5-2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="1 Водитель" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2 Водитель" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="3 Водитель" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -114,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -152,6 +155,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1327,7 +1342,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1425,4 +1440,1107 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>1 Водитель — личный график</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Смена</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Рейсов</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Заработок ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>21.07.2026</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>23.07.2026</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>24.07.2026</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Резерв / ПВЗ</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>25.07.2026</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Сб</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>26.07.2026</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Вс</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>29.07.2026</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>30.07.2026</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>31.07.2026</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>2 Водитель — личный график</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Смена</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Рейсов</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Заработок ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>21.07.2026</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>23.07.2026</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>24.07.2026</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>25.07.2026</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Сб</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>26.07.2026</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Вс</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>29.07.2026</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>30.07.2026</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>31.07.2026</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Резерв / ПВЗ</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>3 Водитель — личный график</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Смена</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Рейсов</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Заработок ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>21.07.2026</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>23.07.2026</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>24.07.2026</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>25.07.2026</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Сб</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>26.07.2026</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Вс</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>02:00 — ночной рейс (Маш.2)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>29.07.2026</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>30.07.2026</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>ВЫХОДНОЙ</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>31.07.2026</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>06:00 — утренний рейс (Маш.1)
+18:00 — вечерний рейс (Маш.1)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>43000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update load times to 01:00, 06:00 and 14:00
Co-authored-by: gltdelete-prog <gltdelete-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SERDECHNOV-grafik-20-31-iyulya-2026.xlsx
+++ b/SERDECHNOV-grafik-20-31-iyulya-2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="1 Водитель" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2 Водитель" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="3 Водитель" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Чек-лист ПВЗ" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -165,6 +166,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -557,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>3 рейса/сутки · 2 машины · 4000 ₽/рейс + 500 ₽ ночная смена · норма 1341 ШК</t>
+          <t>3 рейса/сутки (01:00, 06:00, 14:00) · 2 машины · 4000 ₽/рейс + 500 ₽ ночная смена · норма 1341 ШК</t>
         </is>
       </c>
     </row>
@@ -574,20 +578,20 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>02:00
-(Маш.2)</t>
+          <t>01:00
+(Машина 2)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>06:00
-(Маш.1)</t>
+(Машина 1)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>18:00
-(Маш.1)</t>
+          <t>14:00
+(Машина 1)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1505,8 +1509,8 @@
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
@@ -1529,8 +1533,8 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -1553,8 +1557,8 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -1577,8 +1581,8 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -1680,8 +1684,8 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -1704,7 +1708,7 @@
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -1727,8 +1731,8 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
@@ -1751,8 +1755,8 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -1775,7 +1779,7 @@
       </c>
       <c r="C15" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -1925,7 +1929,7 @@
       </c>
       <c r="C6" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
@@ -1948,7 +1952,7 @@
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -1971,8 +1975,8 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -1995,8 +1999,8 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -2019,8 +2023,8 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -2097,7 +2101,7 @@
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
@@ -2120,7 +2124,7 @@
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -2241,7 +2245,7 @@
       </c>
       <c r="C4" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
@@ -2264,7 +2268,7 @@
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
@@ -2341,7 +2345,7 @@
       </c>
       <c r="C8" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -2364,7 +2368,7 @@
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
@@ -2387,7 +2391,7 @@
       </c>
       <c r="C10" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -2410,7 +2414,7 @@
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Маш.2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
@@ -2433,8 +2437,8 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -2511,8 +2515,8 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>06:00 — утренний рейс (Маш.1)
-18:00 — вечерний рейс (Маш.1)</t>
+          <t>06:00 — утренний рейс (Машина 1)
+14:00 — дневной рейс (Машина 1)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -2535,6 +2539,226 @@
       </c>
       <c r="E16" s="10" t="n">
         <v>43000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Ежедневный чек-лист — маршрут 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Время</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Действие</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Порог ШК</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Машина</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Кто</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Проверить ШК перед ночной загрузкой</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>≥ 1300</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Дежурный ПВЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Загрузка маршрут 7 (ночь)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>1341</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Машина 2</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Ночной водитель</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Проверить ШК перед утренней загрузкой</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>≥ 1300</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Дежурный ПВЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Загрузка маршрут 7 (утро)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>1341</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Машина 1</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Дневной водитель</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Проверить ШК перед дневной загрузкой</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>≥ 1300</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Дежурный ПВЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Загрузка маршрут 7 (день)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>1341</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Машина 1</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Дневной водитель</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>